<commit_message>
Added Python environment setup instructions
</commit_message>
<xml_diff>
--- a/workshop/2022/Agenda/CE-QUAL-W2_Workshop_Aug_2022_Agenda.xlsx
+++ b/workshop/2022/Agenda/CE-QUAL-W2_Workshop_Aug_2022_Agenda.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/todd/GitHub/environmentalsystems/CE-QUAL-W2/workshop/2022/Agenda/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD21511F-ED85-8243-8FC8-3464A7E2427A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0294683D-98CF-BF4C-BF23-B74CD25203A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{5524DC16-E37C-514A-B687-063004997C4D}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="66">
   <si>
     <t>Todd</t>
   </si>
@@ -161,9 +161,6 @@
     <t>Discussion / Tours</t>
   </si>
   <si>
-    <t>Tour - Fish Flume</t>
-  </si>
-  <si>
     <t>Tour - Sediment Lab</t>
   </si>
   <si>
@@ -228,6 +225,18 @@
   </si>
   <si>
     <t>2.09 Case Study - Total Dissolved Gas</t>
+  </si>
+  <si>
+    <t>-- FIRE DRILL &amp; BREAK --</t>
+  </si>
+  <si>
+    <t>Tour - CEERF (Fish Flume):</t>
+  </si>
+  <si>
+    <t>Cognitive Environmental Effects Research Flume</t>
+  </si>
+  <si>
+    <t>3.04 Workshop - Upgrade to V4.5, continued</t>
   </si>
 </sst>
 </file>
@@ -611,7 +620,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -664,9 +673,6 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -721,12 +727,6 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -739,9 +739,6 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
@@ -775,12 +772,15 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -790,13 +790,19 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -883,11 +889,29 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1219,48 +1243,48 @@
     <col min="1" max="1" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="1.33203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="38.83203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5" style="34" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.83203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" style="34" customWidth="1"/>
-    <col min="8" max="8" width="38.83203125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" style="34" customWidth="1"/>
-    <col min="10" max="16384" width="8.83203125" style="24"/>
+    <col min="4" max="4" width="42.83203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5" style="33" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="42.83203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" style="33" customWidth="1"/>
+    <col min="8" max="8" width="42.83203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" style="33" customWidth="1"/>
+    <col min="10" max="16384" width="8.83203125" style="23"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="54" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-    </row>
-    <row r="3" spans="1:9" s="25" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="62" t="s">
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+      <c r="I1" s="54"/>
+    </row>
+    <row r="3" spans="1:9" s="24" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="62" t="s">
+      <c r="B3" s="57"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62" t="s">
+      <c r="E3" s="57"/>
+      <c r="F3" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62" t="s">
+      <c r="G3" s="57"/>
+      <c r="H3" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="62"/>
-    </row>
-    <row r="4" spans="1:9" s="25" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I3" s="57"/>
+    </row>
+    <row r="4" spans="1:9" s="24" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
@@ -1268,19 +1292,19 @@
         <v>10</v>
       </c>
       <c r="C4" s="4"/>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="21" t="s">
         <v>23</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="22" t="s">
+      <c r="F4" s="21" t="s">
         <v>23</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="22" t="s">
+      <c r="H4" s="21" t="s">
         <v>23</v>
       </c>
       <c r="I4" s="9" t="s">
@@ -1294,22 +1318,22 @@
       <c r="B5" s="2">
         <v>0.36458333333333331</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="27" t="s">
+      <c r="E5" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="F5" s="26" t="s">
-        <v>42</v>
-      </c>
-      <c r="G5" s="29" t="s">
+      <c r="F5" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" s="28" t="s">
         <v>3</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="I5" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="I5" s="18" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1320,11 +1344,13 @@
       <c r="B6" s="2">
         <v>0.375</v>
       </c>
-      <c r="D6" s="48"/>
-      <c r="E6" s="42"/>
-      <c r="F6" s="47"/>
-      <c r="G6" s="30"/>
-      <c r="H6" s="43"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="51" t="s">
+        <v>64</v>
+      </c>
       <c r="I6" s="20"/>
     </row>
     <row r="7" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1334,20 +1360,22 @@
       <c r="B7" s="2">
         <v>0.38541666666666702</v>
       </c>
-      <c r="D7" s="26" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" s="27" t="s">
-        <v>0</v>
-      </c>
-      <c r="F7" s="26" t="s">
-        <v>55</v>
-      </c>
-      <c r="G7" s="29" t="s">
+      <c r="D7" s="58" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7" s="59"/>
+      <c r="F7" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="G7" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="H7" s="18"/>
-      <c r="I7" s="20"/>
+      <c r="H7" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="I7" s="18" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="8" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
@@ -1356,11 +1384,11 @@
       <c r="B8" s="2">
         <v>0.39583333333333298</v>
       </c>
-      <c r="D8" s="47"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="47"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="18"/>
+      <c r="D8" s="60"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="43"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="51"/>
       <c r="I8" s="20"/>
     </row>
     <row r="9" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1370,18 +1398,20 @@
       <c r="B9" s="2">
         <v>0.40625</v>
       </c>
-      <c r="D9" s="58" t="s">
+      <c r="D9" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="F9" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="59"/>
-      <c r="F9" s="58" t="s">
+      <c r="G9" s="56"/>
+      <c r="H9" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="G9" s="59"/>
-      <c r="H9" s="58" t="s">
-        <v>4</v>
-      </c>
-      <c r="I9" s="59"/>
+      <c r="I9" s="56"/>
     </row>
     <row r="10" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
@@ -1390,22 +1420,18 @@
       <c r="B10" s="2">
         <v>0.41666666666666702</v>
       </c>
-      <c r="D10" s="26" t="s">
-        <v>34</v>
-      </c>
-      <c r="E10" s="27" t="s">
-        <v>5</v>
-      </c>
+      <c r="D10" s="43"/>
+      <c r="E10" s="27"/>
       <c r="F10" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="H10" s="45" t="s">
-        <v>47</v>
-      </c>
-      <c r="I10" s="46" t="s">
+      <c r="H10" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="I10" s="42" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1416,12 +1442,16 @@
       <c r="B11" s="2">
         <v>0.42708333333333298</v>
       </c>
-      <c r="D11" s="44"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="33"/>
+      <c r="D11" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="F11" s="22"/>
+      <c r="G11" s="32"/>
       <c r="H11" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I11" s="13" t="s">
         <v>6</v>
@@ -1434,16 +1464,12 @@
       <c r="B12" s="2">
         <v>0.4375</v>
       </c>
-      <c r="D12" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="E12" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="F12" s="45" t="s">
-        <v>57</v>
-      </c>
-      <c r="G12" s="46" t="s">
+      <c r="D12" s="40"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="41" t="s">
+        <v>56</v>
+      </c>
+      <c r="G12" s="42" t="s">
         <v>5</v>
       </c>
       <c r="H12" s="12"/>
@@ -1456,18 +1482,22 @@
       <c r="B13" s="2">
         <v>0.44791666666666702</v>
       </c>
-      <c r="D13" s="44"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="53" t="s">
-        <v>58</v>
-      </c>
-      <c r="G13" s="54" t="s">
+      <c r="D13" s="55" t="s">
+        <v>4</v>
+      </c>
+      <c r="E13" s="56"/>
+      <c r="F13" s="49" t="s">
+        <v>57</v>
+      </c>
+      <c r="G13" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="H13" s="58" t="s">
-        <v>4</v>
-      </c>
-      <c r="I13" s="59"/>
+      <c r="H13" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="I13" s="28" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="14" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
@@ -1476,20 +1506,20 @@
       <c r="B14" s="2">
         <v>0.45833333333333298</v>
       </c>
-      <c r="D14" s="60" t="s">
+      <c r="D14" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="E14" s="61"/>
-      <c r="F14" s="58" t="s">
+      <c r="G14" s="56"/>
+      <c r="H14" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="G14" s="59"/>
-      <c r="H14" s="55" t="s">
-        <v>41</v>
-      </c>
-      <c r="I14" s="19" t="s">
-        <v>8</v>
-      </c>
+      <c r="I14" s="56"/>
     </row>
     <row r="15" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
@@ -1498,20 +1528,20 @@
       <c r="B15" s="2">
         <v>0.46875</v>
       </c>
-      <c r="D15" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="E15" s="27" t="s">
+      <c r="D15" s="40"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="41" t="s">
+        <v>58</v>
+      </c>
+      <c r="G15" s="42" t="s">
+        <v>6</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="I15" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="F15" s="45" t="s">
-        <v>59</v>
-      </c>
-      <c r="G15" s="46" t="s">
-        <v>6</v>
-      </c>
-      <c r="H15" s="56"/>
-      <c r="I15" s="21"/>
     </row>
     <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
@@ -1520,20 +1550,20 @@
       <c r="B16" s="2">
         <v>0.47916666666666702</v>
       </c>
-      <c r="D16" s="44"/>
-      <c r="E16" s="28"/>
+      <c r="D16" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" s="26" t="s">
+        <v>3</v>
+      </c>
       <c r="F16" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G16" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="H16" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="I16" s="29" t="s">
-        <v>3</v>
-      </c>
+      <c r="H16" s="12"/>
+      <c r="I16" s="15"/>
     </row>
     <row r="17" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
@@ -1542,23 +1572,19 @@
       <c r="B17" s="2">
         <v>0.48958333333333298</v>
       </c>
-      <c r="D17" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="F17" s="45" t="s">
-        <v>61</v>
-      </c>
-      <c r="G17" s="46" t="s">
+      <c r="D17" s="40"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="41" t="s">
+        <v>60</v>
+      </c>
+      <c r="G17" s="42" t="s">
         <v>3</v>
       </c>
       <c r="H17" s="11" t="s">
         <v>50</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1568,16 +1594,18 @@
       <c r="B18" s="2">
         <v>0.5</v>
       </c>
-      <c r="D18" s="12"/>
-      <c r="E18" s="51"/>
-      <c r="F18" s="53" t="s">
-        <v>62</v>
-      </c>
-      <c r="G18" s="54" t="s">
+      <c r="D18" s="90" t="s">
+        <v>22</v>
+      </c>
+      <c r="E18" s="91"/>
+      <c r="F18" s="49" t="s">
+        <v>61</v>
+      </c>
+      <c r="G18" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="H18" s="12"/>
-      <c r="I18" s="15"/>
+      <c r="H18" s="45"/>
+      <c r="I18" s="14"/>
     </row>
     <row r="19" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
@@ -1586,18 +1614,16 @@
       <c r="B19" s="2">
         <v>0.51041666666666696</v>
       </c>
-      <c r="D19" s="91" t="s">
+      <c r="D19" s="92"/>
+      <c r="E19" s="93"/>
+      <c r="F19" s="81" t="s">
         <v>22</v>
       </c>
-      <c r="E19" s="92"/>
-      <c r="F19" s="82" t="s">
+      <c r="G19" s="82"/>
+      <c r="H19" s="81" t="s">
         <v>22</v>
       </c>
-      <c r="G19" s="83"/>
-      <c r="H19" s="82" t="s">
-        <v>22</v>
-      </c>
-      <c r="I19" s="83"/>
+      <c r="I19" s="82"/>
     </row>
     <row r="20" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
@@ -1606,12 +1632,12 @@
       <c r="B20" s="2">
         <v>0.52083333333333304</v>
       </c>
-      <c r="D20" s="91"/>
-      <c r="E20" s="92"/>
-      <c r="F20" s="84"/>
-      <c r="G20" s="85"/>
-      <c r="H20" s="84"/>
-      <c r="I20" s="85"/>
+      <c r="D20" s="92"/>
+      <c r="E20" s="93"/>
+      <c r="F20" s="83"/>
+      <c r="G20" s="84"/>
+      <c r="H20" s="83"/>
+      <c r="I20" s="84"/>
     </row>
     <row r="21" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
@@ -1620,12 +1646,12 @@
       <c r="B21" s="2">
         <v>0.53125</v>
       </c>
-      <c r="D21" s="91"/>
-      <c r="E21" s="92"/>
-      <c r="F21" s="84"/>
-      <c r="G21" s="85"/>
-      <c r="H21" s="84"/>
-      <c r="I21" s="85"/>
+      <c r="D21" s="92"/>
+      <c r="E21" s="93"/>
+      <c r="F21" s="83"/>
+      <c r="G21" s="84"/>
+      <c r="H21" s="83"/>
+      <c r="I21" s="84"/>
     </row>
     <row r="22" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
@@ -1634,12 +1660,12 @@
       <c r="B22" s="2">
         <v>0.54166666666666696</v>
       </c>
-      <c r="D22" s="91"/>
-      <c r="E22" s="92"/>
-      <c r="F22" s="84"/>
-      <c r="G22" s="85"/>
-      <c r="H22" s="84"/>
-      <c r="I22" s="85"/>
+      <c r="D22" s="92"/>
+      <c r="E22" s="93"/>
+      <c r="F22" s="83"/>
+      <c r="G22" s="84"/>
+      <c r="H22" s="83"/>
+      <c r="I22" s="84"/>
     </row>
     <row r="23" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
@@ -1648,12 +1674,12 @@
       <c r="B23" s="2">
         <v>0.55208333333333304</v>
       </c>
-      <c r="D23" s="91"/>
-      <c r="E23" s="92"/>
-      <c r="F23" s="84"/>
-      <c r="G23" s="85"/>
-      <c r="H23" s="84"/>
-      <c r="I23" s="85"/>
+      <c r="D23" s="94"/>
+      <c r="E23" s="95"/>
+      <c r="F23" s="83"/>
+      <c r="G23" s="84"/>
+      <c r="H23" s="83"/>
+      <c r="I23" s="84"/>
     </row>
     <row r="24" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
@@ -1662,12 +1688,16 @@
       <c r="B24" s="2">
         <v>0.5625</v>
       </c>
-      <c r="D24" s="91"/>
-      <c r="E24" s="92"/>
-      <c r="F24" s="86"/>
-      <c r="G24" s="87"/>
-      <c r="H24" s="86"/>
-      <c r="I24" s="87"/>
+      <c r="D24" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="F24" s="85"/>
+      <c r="G24" s="86"/>
+      <c r="H24" s="85"/>
+      <c r="I24" s="86"/>
     </row>
     <row r="25" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
@@ -1676,20 +1706,16 @@
       <c r="B25" s="2">
         <v>0.57291666666666696</v>
       </c>
-      <c r="D25" s="26" t="s">
-        <v>31</v>
-      </c>
-      <c r="E25" s="29" t="s">
-        <v>6</v>
-      </c>
-      <c r="F25" s="26" t="s">
-        <v>43</v>
-      </c>
-      <c r="G25" s="29" t="s">
+      <c r="D25" s="12"/>
+      <c r="E25" s="47"/>
+      <c r="F25" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="G25" s="28" t="s">
         <v>5</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="I25" s="13" t="s">
         <v>7</v>
@@ -1702,12 +1728,16 @@
       <c r="B26" s="2">
         <v>0.58333333333333304</v>
       </c>
-      <c r="D26" s="47"/>
-      <c r="E26" s="30"/>
-      <c r="F26" s="48"/>
-      <c r="G26" s="39"/>
-      <c r="H26" s="49"/>
-      <c r="I26" s="14"/>
+      <c r="D26" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="E26" s="28" t="s">
+        <v>6</v>
+      </c>
+      <c r="F26" s="44"/>
+      <c r="G26" s="36"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="15"/>
     </row>
     <row r="27" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
@@ -1716,20 +1746,20 @@
       <c r="B27" s="2">
         <v>0.59375</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E27" s="10" t="s">
-        <v>6</v>
-      </c>
+      <c r="D27" s="43"/>
+      <c r="E27" s="29"/>
       <c r="F27" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G27" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="H27" s="37"/>
-      <c r="I27" s="14"/>
+      <c r="H27" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="I27" s="13" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
@@ -1738,12 +1768,14 @@
       <c r="B28" s="2">
         <v>0.60416666666666696</v>
       </c>
-      <c r="D28" s="23"/>
-      <c r="E28" s="33"/>
+      <c r="D28" s="55" t="s">
+        <v>4</v>
+      </c>
+      <c r="E28" s="56"/>
       <c r="F28" s="12"/>
       <c r="G28" s="15"/>
-      <c r="H28" s="38"/>
-      <c r="I28" s="15"/>
+      <c r="H28" s="45"/>
+      <c r="I28" s="14"/>
     </row>
     <row r="29" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
@@ -1752,18 +1784,18 @@
       <c r="B29" s="2">
         <v>0.61458333333333304</v>
       </c>
-      <c r="D29" s="58" t="s">
+      <c r="D29" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="F29" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="E29" s="59"/>
-      <c r="F29" s="58" t="s">
-        <v>4</v>
-      </c>
-      <c r="G29" s="59"/>
-      <c r="H29" s="90" t="s">
-        <v>4</v>
-      </c>
-      <c r="I29" s="59"/>
+      <c r="G29" s="56"/>
+      <c r="H29" s="45"/>
+      <c r="I29" s="14"/>
     </row>
     <row r="30" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
@@ -1772,24 +1804,16 @@
       <c r="B30" s="2">
         <v>0.625</v>
       </c>
-      <c r="D30" s="26" t="s">
-        <v>29</v>
-      </c>
-      <c r="E30" s="29" t="s">
-        <v>54</v>
-      </c>
-      <c r="F30" s="40" t="s">
-        <v>45</v>
-      </c>
-      <c r="G30" s="29" t="s">
+      <c r="D30" s="22"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="37" t="s">
+        <v>44</v>
+      </c>
+      <c r="G30" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="H30" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="I30" s="13" t="s">
-        <v>0</v>
-      </c>
+      <c r="H30" s="12"/>
+      <c r="I30" s="15"/>
     </row>
     <row r="31" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
@@ -1798,12 +1822,18 @@
       <c r="B31" s="2">
         <v>0.63541666666666696</v>
       </c>
-      <c r="D31" s="47"/>
-      <c r="E31" s="30"/>
-      <c r="F31" s="50"/>
-      <c r="G31" s="30"/>
-      <c r="H31" s="49"/>
-      <c r="I31" s="14"/>
+      <c r="D31" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="E31" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="F31" s="46"/>
+      <c r="G31" s="29"/>
+      <c r="H31" s="58" t="s">
+        <v>4</v>
+      </c>
+      <c r="I31" s="59"/>
     </row>
     <row r="32" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
@@ -1812,20 +1842,20 @@
       <c r="B32" s="2">
         <v>0.64583333333333304</v>
       </c>
-      <c r="D32" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E32" s="10" t="s">
-        <v>53</v>
-      </c>
+      <c r="D32" s="43"/>
+      <c r="E32" s="29"/>
       <c r="F32" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="G32" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="G32" s="96" t="s">
         <v>2</v>
       </c>
-      <c r="H32" s="12"/>
-      <c r="I32" s="15"/>
+      <c r="H32" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="I32" s="18" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="33" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
@@ -1834,14 +1864,14 @@
       <c r="B33" s="2">
         <v>0.65625</v>
       </c>
-      <c r="D33" s="23"/>
-      <c r="E33" s="33"/>
+      <c r="D33" s="55" t="s">
+        <v>4</v>
+      </c>
+      <c r="E33" s="56"/>
       <c r="F33" s="12"/>
-      <c r="G33" s="15"/>
-      <c r="H33" s="90" t="s">
-        <v>4</v>
-      </c>
-      <c r="I33" s="59"/>
+      <c r="G33" s="47"/>
+      <c r="H33" s="97"/>
+      <c r="I33" s="19"/>
     </row>
     <row r="34" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
@@ -1850,20 +1880,18 @@
       <c r="B34" s="2">
         <v>0.66666666666666696</v>
       </c>
-      <c r="D34" s="58" t="s">
+      <c r="D34" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F34" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="E34" s="59"/>
-      <c r="F34" s="58" t="s">
-        <v>4</v>
-      </c>
-      <c r="G34" s="59"/>
-      <c r="H34" s="31" t="s">
-        <v>1</v>
-      </c>
-      <c r="I34" s="19" t="s">
-        <v>0</v>
-      </c>
+      <c r="G34" s="89"/>
+      <c r="H34" s="31"/>
+      <c r="I34" s="20"/>
     </row>
     <row r="35" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
@@ -1872,22 +1900,18 @@
       <c r="B35" s="2">
         <v>0.67708333333333404</v>
       </c>
-      <c r="D35" s="31" t="s">
+      <c r="D35" s="22"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="E35" s="19" t="s">
+      <c r="G35" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="F35" s="41" t="s">
-        <v>21</v>
-      </c>
-      <c r="G35" s="52" t="s">
-        <v>0</v>
-      </c>
-      <c r="H35" s="31" t="s">
+      <c r="H35" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="I35" s="19" t="s">
+      <c r="I35" s="18" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1898,12 +1922,16 @@
       <c r="B36" s="2">
         <v>0.6875</v>
       </c>
-      <c r="D36" s="32"/>
-      <c r="E36" s="21"/>
-      <c r="F36" s="36"/>
-      <c r="G36" s="35"/>
-      <c r="H36" s="32"/>
-      <c r="I36" s="21"/>
+      <c r="D36" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="E36" s="53" t="s">
+        <v>0</v>
+      </c>
+      <c r="F36" s="35"/>
+      <c r="G36" s="34"/>
+      <c r="H36" s="31"/>
+      <c r="I36" s="20"/>
     </row>
     <row r="37" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
@@ -1913,89 +1941,87 @@
       <c r="A38" s="5"/>
       <c r="B38" s="5"/>
       <c r="C38" s="7"/>
-      <c r="H38" s="65" t="s">
+      <c r="H38" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="I38" s="65"/>
+      <c r="I38" s="64"/>
     </row>
     <row r="39" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="6"/>
       <c r="B39" s="6"/>
       <c r="C39" s="8"/>
-      <c r="D39" s="66" t="s">
+      <c r="D39" s="65" t="s">
         <v>26</v>
       </c>
-      <c r="E39" s="67"/>
-      <c r="F39" s="34"/>
-      <c r="H39" s="72" t="s">
+      <c r="E39" s="66"/>
+      <c r="F39" s="33"/>
+      <c r="H39" s="71" t="s">
         <v>18</v>
       </c>
-      <c r="I39" s="73"/>
+      <c r="I39" s="72"/>
     </row>
     <row r="40" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
-      <c r="D40" s="68"/>
-      <c r="E40" s="69"/>
-      <c r="H40" s="74" t="s">
+      <c r="D40" s="67"/>
+      <c r="E40" s="68"/>
+      <c r="H40" s="73" t="s">
         <v>24</v>
       </c>
-      <c r="I40" s="75"/>
+      <c r="I40" s="74"/>
     </row>
     <row r="41" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
-      <c r="D41" s="68"/>
-      <c r="E41" s="69"/>
-      <c r="H41" s="76" t="s">
+      <c r="D41" s="67"/>
+      <c r="E41" s="68"/>
+      <c r="H41" s="75" t="s">
         <v>25</v>
       </c>
-      <c r="I41" s="77"/>
+      <c r="I41" s="76"/>
     </row>
     <row r="42" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
-      <c r="D42" s="68"/>
-      <c r="E42" s="69"/>
-      <c r="H42" s="88" t="s">
+      <c r="D42" s="67"/>
+      <c r="E42" s="68"/>
+      <c r="H42" s="87" t="s">
         <v>39</v>
       </c>
-      <c r="I42" s="89"/>
+      <c r="I42" s="88"/>
     </row>
     <row r="43" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D43" s="68"/>
-      <c r="E43" s="69"/>
-      <c r="H43" s="63" t="s">
+      <c r="D43" s="67"/>
+      <c r="E43" s="68"/>
+      <c r="H43" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="I43" s="64"/>
+      <c r="I43" s="63"/>
     </row>
     <row r="44" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D44" s="68"/>
-      <c r="E44" s="69"/>
-      <c r="H44" s="78" t="s">
+      <c r="D44" s="67"/>
+      <c r="E44" s="68"/>
+      <c r="H44" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="I44" s="79"/>
+      <c r="I44" s="78"/>
     </row>
     <row r="45" spans="1:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D45" s="70"/>
-      <c r="E45" s="71"/>
-      <c r="H45" s="80" t="s">
+      <c r="D45" s="69"/>
+      <c r="E45" s="70"/>
+      <c r="H45" s="79" t="s">
         <v>16</v>
       </c>
-      <c r="I45" s="81"/>
+      <c r="I45" s="80"/>
     </row>
   </sheetData>
-  <mergeCells count="29">
-    <mergeCell ref="H19:I24"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="H29:I29"/>
+  <mergeCells count="28">
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="H14:I14"/>
     <mergeCell ref="F29:G29"/>
-    <mergeCell ref="D19:E24"/>
     <mergeCell ref="F19:G24"/>
+    <mergeCell ref="D18:E23"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D7:E8"/>
+    <mergeCell ref="D13:E13"/>
     <mergeCell ref="H43:I43"/>
     <mergeCell ref="H38:I38"/>
     <mergeCell ref="D39:E45"/>
@@ -2004,19 +2030,20 @@
     <mergeCell ref="H41:I41"/>
     <mergeCell ref="H44:I44"/>
     <mergeCell ref="H45:I45"/>
+    <mergeCell ref="H19:I24"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="F34:G34"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D14:E14"/>
     <mergeCell ref="F9:G9"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="H3:I3"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H13:I13"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="68" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup scale="63" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>